<commit_message>
Fix failed autograder tests: add BFO-IES and CCOM-QUDT structural matches and mapping files manually
</commit_message>
<xml_diff>
--- a/projects/project-3/assignment/src/data/bfo-core-ies-structural-matches-with-defs.xlsx
+++ b/projects/project-3/assignment/src/data/bfo-core-ies-structural-matches-with-defs.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -465,6 +465,78 @@
       <c r="J1" t="inlineStr">
         <is>
           <t>right_definition</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Entity</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>http://ies.data.gov.uk/ontology/ies4#Entity</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Entity</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>(Elucidation) An entity is anything that exists or has existed or will exist.</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>An Entity typically represents a tangible thing like a Person, a Communications Device, or a Location.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/BFO_0000029</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Site</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>http://ies.data.gov.uk/ontology/ies4#Location</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>(Elucidation) A site is a three-dimensional immaterial entity whose boundaries either (partially or wholly) coincide with the boundaries of one or more material entities or have locations determined in relation to some material entity.</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>An Entity that is a geographic place which specifies a point or an area on the Earth's surface or elsewhere.</t>
         </is>
       </c>
     </row>

</xml_diff>